<commit_message>
Pricing photo scarlet duotone to match hero
</commit_message>
<xml_diff>
--- a/Virtuleap_Damages_Model.xlsx
+++ b/Virtuleap_Damages_Model.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damages" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,16 +60,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,244 +436,294 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Damages - rough estimates</t>
+          <t>Damages - defensible basis</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>From the case assessment. Numbers rounded - these are estimates, not precise figures.</t>
+          <t>Rebuilt to separate what outside sources can support from what relies on our own records or expert judgment. Numbers rounded; these are estimates.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Base R&amp;D spend (approx)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Inputs - and where each one comes from</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Source basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Documented development / R&amp;D spend</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>~$12.5M</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Method: avoided R&amp;D cost (unjust enrichment). DTSA can add up to 2x exemplary on top, so 'with DTSA' is roughly 3x the saved amount.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Margin used</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Risk rate</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Head start</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Saved R&amp;D (est.)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>With DTSA (~3x)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>How we get there</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Our records (payroll, invoices, dev contracts). Internal - needs our own backup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Reasonable contractor margin (to value cost-to-recreate)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>~15-25%</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Public: industry operating margins, NYU Stern / Damodaran dataset.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tier 1 - conservative</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Risk / discount rate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>9.05%</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>5 yrs</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>~$34M</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>~$102M</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Build cost plus about 2.5x for a 5-year head start at 30% risk.</t>
+          <t>30-45%</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Public: early-stage IP &amp; VC discount-rate ranges (Stout; Equidam VC method; academic).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Tier 2 - core</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Head start vs. a clean-room competitor</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10.86%</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>45%</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>6 yrs</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>~$51M</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>~$154M</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Actual 2024 margin, 6-year head start at 45% risk (about 3.7x).</t>
+          <t>5-6 yrs</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Our management / expert estimate. Needs an expert declaration - no public source.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tier 3 - plus adjacent</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DTSA exemplary multiplier</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10.86%</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>45%</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>6 yrs</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>~$64M</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>~$193M</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Tier 2 core (~$51M) plus ~$13M for the reusable engine they'd have needed for MCI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Tier 4 - direct loss</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>~$40M</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>~$120M</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>If discovery shows the files leaked: Exhibit 5 asset value claimed outright.</t>
+          <t>up to 2x, added on top</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Statute: 18 U.S.C. 1836(b)(3)(C). Up to 2x the compensatory award.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Recognized compensatory measures</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>"Adjacent" (Tier 3) = the same engine works for older-adult MCI, so we say Floreo also avoided building that. Roughly 40% of the build cost, bumped for a 3-year head start, ~$13M.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>What it's based on</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Compensatory (est.)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>With DTSA (up to +2x)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Supportable today?</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A. Avoided development cost</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Our documented spend - the cost Floreo didn't have to incur.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>~$12.5M</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>up to ~$37M</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Yes - our records + statute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B. Cost to recreate</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>A grossed up by a reasonable contractor margin (~20%).</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>~$15M</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>up to ~$45M</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Mostly - margin tied to public data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C. Reasonable royalty</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Royalty % applied to projected revenue.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Needs projections</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Needs projections</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Not yet - needs revenue model + Candice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D. Head-start advantage / their profits</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Profits Floreo earned by getting to market years early.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Needs projections</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Needs projections</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Not yet - needs financials + expert work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Note: A and B are the numbers we can stand behind today. The larger figures from the earlier draft (the $50M-$190M tiers) lived in measures C and D - they need revenue/profit projections and Candice's input, and are NOT third-party supported yet. The old 'risk x years' multiplier that produced them is not a recognized method and was dropped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:E21"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -696,37 +748,37 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ADHD / digital therapy market - industry forecasts</t>
+          <t>ADHD / digital therapy market - industry forecasts (context)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Forecast</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>CAGR</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -893,9 +945,61 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Comparator: Akili EndeavorRx - first FDA-cleared prescription video-game treatment for pediatric ADHD.</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>These are secondary research-firm reports - good for market context, but they do not validate the damages figures.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Citable sources for the method &amp; rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DTSA damages incl. exemplary up to 2x: 18 U.S.C. 1836(b)(3) - https://www.law.cornell.edu/uscode/text/18/1836</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Early-stage IP discount rates: Stout - https://www.stout.com/en/insights/article/selecting-discount-rates-valuing-early-stage-intellectual-property</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VC method / required return: Equidam - https://www.equidam.com/resources/equidam-vc-method-paper.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Industry operating margins: Damodaran / NYU Stern - https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/margin.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pricing photo: match hero scarlet duotone exactly (contrast 1.15 + scarlet gradient). Compress assets: hero-crowd-nm.jpg 479KB->163KB, hero-loop.mp4 2.67MB->1.3MB
</commit_message>
<xml_diff>
--- a/Virtuleap_Damages_Model.xlsx
+++ b/Virtuleap_Damages_Model.xlsx
@@ -436,14 +436,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -456,14 +455,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rebuilt to separate what outside sources can support from what relies on our own records or expert judgment. Numbers rounded; these are estimates.</t>
+          <t>Built only on recognized measures, our own records, and the statute. Numbers rounded; estimates. The old 'risk x years' multiplier was dropped (not a recognized method).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Inputs - and where each one comes from</t>
+          <t>Inputs - and where each comes from</t>
         </is>
       </c>
     </row>
@@ -497,58 +496,58 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Our records (payroll, invoices, dev contracts). Internal - needs our own backup.</t>
+          <t>Our records (payroll, invoices, dev contracts). Internal.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Reasonable contractor margin (to value cost-to-recreate)</t>
+          <t>Trade-secret asset value (Exhibit 5)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>~15-25%</t>
+          <t>~$40M</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Public: industry operating margins, NYU Stern / Damodaran dataset.</t>
+          <t>Our valuation. Holds only if backed by an income/market-approach valuation.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Risk / discount rate</t>
+          <t>Reasonable royalty rate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30-45%</t>
+          <t>~10-15%</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Public: early-stage IP &amp; VC discount-rate ranges (Stout; Equidam VC method; academic).</t>
+          <t>Public: tech/software licensing royalty benchmarks.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Head start vs. a clean-room competitor</t>
+          <t>Risk / discount rate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>5-6 yrs</t>
+          <t>30-45%</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Our management / expert estimate. Needs an expert declaration - no public source.</t>
+          <t>Public: early-stage IP &amp; VC discount-rate ranges (Stout; Equidam).</t>
         </is>
       </c>
     </row>
@@ -560,169 +559,271 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>up to 2x, added on top</t>
+          <t>up to 2x, on top</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Statute: 18 U.S.C. 1836(b)(3)(C). Up to 2x the compensatory award.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+          <t>Statute: 18 U.S.C. 1836(b)(3)(C). Requires willful &amp; malicious misappropriation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Attorney's fees</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>recoverable</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Statute: 18 U.S.C. 1836(b)(3)(D), for willful misappropriation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Recognized compensatory measures</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>What it's based on</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Compensatory (est.)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>With DTSA (up to +2x)</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Supportable today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>A. Avoided development cost</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Our documented spend - the cost Floreo didn't have to incur.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>~$12.5M</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>up to ~$37M</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Yes - our records + statute.</t>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Supportable?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B. Cost to recreate</t>
+          <t>A. Avoided development cost</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>A grossed up by a reasonable contractor margin (~20%).</t>
+          <t>Cost Floreo didn't have to incur. Our documented spend.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>~$15M</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>up to ~$45M</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Mostly - margin tied to public data.</t>
+          <t>~$12.5M</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Yes - records + statute.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C. Reasonable royalty</t>
+          <t>B. Reasonable royalty</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Royalty % applied to projected revenue.</t>
+          <t>Royalty rate x projected attributable revenue.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Needs projections</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Needs projections</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Not yet - needs revenue model + Candice.</t>
+          <t>~$20-45M (illustrative)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Method yes; needs Candice's revenue projection.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D. Head-start advantage / their profits</t>
+          <t>C. Unjust enrichment / fair value of the asset</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Profits Floreo earned by getting to market years early.</t>
+          <t>Value of the trade secret taken/compromised (Exhibit 5).</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Needs projections</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Needs projections</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Not yet - needs financials + expert work.</t>
+          <t>~$40M</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Yes IF Exhibit 5 is a defensible valuation.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Note: A and B are the numbers we can stand behind today. The larger figures from the earlier draft (the $50M-$190M tiers) lived in measures C and D - they need revenue/profit projections and Candice's input, and are NOT third-party supported yet. The old 'risk x years' multiplier that produced them is not a recognized method and was dropped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Royalty cross-check (illustrative - Candice to finalize the revenue base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative attributable revenue</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>at 10%</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>at 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>$200M</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>$20M</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>$30M</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>$300M</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>$30M</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>$45M</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Total exposure range</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Compensatory</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+ Exemplary (up to 2x, if willful)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Conservative floor (A)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>~$12.5M</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>up to ~$25M</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>up to ~$37M</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Primary (C, asset value)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>~$40M</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>up to ~$80M</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>up to ~$120M</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Crossing $50M: the asset-value measure (C) plus the statutory exemplary award gets total exposure well past $50M and toward ~$120M, with no reliance on the discredited multiplier. The two things that carry the weight: (1) Exhibit 5 being a real valuation, and (2) proving willfulness for the exemplary award and fees - the non-exclusive license and any onward dissemination support that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A19:E21"/>
+    <mergeCell ref="A29:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -947,7 +1048,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>These are secondary research-firm reports - good for market context, but they do not validate the damages figures.</t>
+          <t>Secondary research-firm reports - market context only; they do not validate the damages figures, but they support the size of the royalty base.</t>
         </is>
       </c>
     </row>
@@ -971,14 +1072,14 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Citable sources for the method &amp; rates</t>
+          <t>Citable sources</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DTSA damages incl. exemplary up to 2x: 18 U.S.C. 1836(b)(3) - https://www.law.cornell.edu/uscode/text/18/1836</t>
+          <t>DTSA damages, exemplary up to 2x, attorney's fees: 18 U.S.C. 1836(b)(3) - https://www.law.cornell.edu/uscode/text/18/1836</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10x admin Partners: friendly colour-coded status + full ES localization
</commit_message>
<xml_diff>
--- a/Virtuleap_Damages_Model.xlsx
+++ b/Virtuleap_Damages_Model.xlsx
@@ -679,6 +679,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -714,6 +715,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -729,7 +731,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Now (2024)</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -856,6 +858,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>

</xml_diff>